<commit_message>
Refresh CIL docs and results
</commit_message>
<xml_diff>
--- a/CIL_Results.xlsx
+++ b/CIL_Results.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="14725"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="14725" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="seed1993" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,116 +15,6 @@
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="35">
-  <si>
-    <t>Method</t>
-  </si>
-  <si>
-    <t>CIFAR100 (T=10)</t>
-  </si>
-  <si>
-    <t>CUB200 (T=10)</t>
-  </si>
-  <si>
-    <t>ImageNet-R (T=5)</t>
-  </si>
-  <si>
-    <t>OmniBenchmark (T=10)</t>
-  </si>
-  <si>
-    <t>VTAB (T=5)</t>
-  </si>
-  <si>
-    <t>A_L</t>
-  </si>
-  <si>
-    <t>Ā</t>
-  </si>
-  <si>
-    <t>Full Fine-Tuning</t>
-  </si>
-  <si>
-    <t>SimpleCIL</t>
-  </si>
-  <si>
-    <t>IJCV 2024</t>
-  </si>
-  <si>
-    <t>APER</t>
-  </si>
-  <si>
-    <t>L2P</t>
-  </si>
-  <si>
-    <t>CVPR 2022</t>
-  </si>
-  <si>
-    <t>DualPrompt</t>
-  </si>
-  <si>
-    <t>ECCV 2022</t>
-  </si>
-  <si>
-    <t>CODA-Prompt</t>
-  </si>
-  <si>
-    <t>CVPR 2023</t>
-  </si>
-  <si>
-    <t>LAE</t>
-  </si>
-  <si>
-    <t>ICCV 2023</t>
-  </si>
-  <si>
-    <t>InfLoRA</t>
-  </si>
-  <si>
-    <t>CVPR 2024</t>
-  </si>
-  <si>
-    <t>EASE</t>
-  </si>
-  <si>
-    <t>BiLoRA</t>
-  </si>
-  <si>
-    <t>CVPR 2025</t>
-  </si>
-  <si>
-    <t>SD-LoRA</t>
-  </si>
-  <si>
-    <t>ICLR 2025</t>
-  </si>
-  <si>
-    <t>CL-LoRA</t>
-  </si>
-  <si>
-    <t>iCaRL</t>
-  </si>
-  <si>
-    <t>CVPR 2017</t>
-  </si>
-  <si>
-    <t>Memory</t>
-  </si>
-  <si>
-    <t>FOSTER</t>
-  </si>
-  <si>
-    <t>ImageNet-R (T=10)</t>
-  </si>
-  <si>
-    <t>ImageNet-R (T=20)</t>
-  </si>
-  <si>
-    <t>ImageNet-R (T=40)</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -833,280 +723,280 @@
     </border>
   </borders>
   <cellStyleXfs count="50">
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="7" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="8" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="11" fillId="9" fontId="6" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="11" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="12" fillId="0" fontId="12" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="12" fillId="0" fontId="13" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="13" fillId="0" fontId="14" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="14" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="14" fillId="10" fontId="15" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="15" fillId="11" fontId="16" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="14" fillId="11" fontId="17" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="16" fillId="12" fontId="18" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="17" fillId="0" fontId="19" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="18" fillId="0" fontId="20" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="13" fontId="21" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="14" fontId="22" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="15" fontId="23" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="16" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="17" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="18" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="19" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="20" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="21" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="22" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="23" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="24" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="25" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="26" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="27" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="28" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="29" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="30" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="31" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="32" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="33" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="34" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="35" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="36" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="37" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="38" fontId="25" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="39" fontId="24" numFmtId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="11" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="14" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="15" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="14" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="16" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="17" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="39" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="27">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="49"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="2" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf applyAlignment="1" borderId="0" fillId="3" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="3" fillId="3" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="4" fillId="3" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="4" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="6" fillId="0" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="6" fillId="4" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="7" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="8" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="9" fillId="3" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="5" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="6" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="7" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="6" fillId="8" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="6" fillId="7" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="8" fontId="2" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="2" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="7" fontId="3" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="3" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="10" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="5" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf applyAlignment="1" borderId="5" fillId="4" fontId="5" numFmtId="2" pivotButton="0" quotePrefix="0" xfId="49">
+    <xf numFmtId="2" fontId="5" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="50">
-    <cellStyle builtinId="0" name="常规" xfId="0"/>
-    <cellStyle builtinId="3" name="千位分隔" xfId="1"/>
-    <cellStyle builtinId="4" name="货币" xfId="2"/>
-    <cellStyle builtinId="5" name="百分比" xfId="3"/>
-    <cellStyle builtinId="6" name="千位分隔[0]" xfId="4"/>
-    <cellStyle builtinId="7" name="货币[0]" xfId="5"/>
-    <cellStyle builtinId="8" name="超链接" xfId="6"/>
-    <cellStyle builtinId="9" name="已访问的超链接" xfId="7"/>
-    <cellStyle builtinId="10" name="注释" xfId="8"/>
-    <cellStyle builtinId="11" name="警告文本" xfId="9"/>
-    <cellStyle builtinId="15" name="标题" xfId="10"/>
-    <cellStyle builtinId="53" name="解释性文本" xfId="11"/>
-    <cellStyle builtinId="16" name="标题 1" xfId="12"/>
-    <cellStyle builtinId="17" name="标题 2" xfId="13"/>
-    <cellStyle builtinId="18" name="标题 3" xfId="14"/>
-    <cellStyle builtinId="19" name="标题 4" xfId="15"/>
-    <cellStyle builtinId="20" name="输入" xfId="16"/>
-    <cellStyle builtinId="21" name="输出" xfId="17"/>
-    <cellStyle builtinId="22" name="计算" xfId="18"/>
-    <cellStyle builtinId="23" name="检查单元格" xfId="19"/>
-    <cellStyle builtinId="24" name="链接单元格" xfId="20"/>
-    <cellStyle builtinId="25" name="汇总" xfId="21"/>
-    <cellStyle builtinId="26" name="好" xfId="22"/>
-    <cellStyle builtinId="27" name="差" xfId="23"/>
-    <cellStyle builtinId="28" name="适中" xfId="24"/>
-    <cellStyle builtinId="29" name="强调文字颜色 1" xfId="25"/>
-    <cellStyle builtinId="30" name="20% - 强调文字颜色 1" xfId="26"/>
-    <cellStyle builtinId="31" name="40% - 强调文字颜色 1" xfId="27"/>
-    <cellStyle builtinId="32" name="60% - 强调文字颜色 1" xfId="28"/>
-    <cellStyle builtinId="33" name="强调文字颜色 2" xfId="29"/>
-    <cellStyle builtinId="34" name="20% - 强调文字颜色 2" xfId="30"/>
-    <cellStyle builtinId="35" name="40% - 强调文字颜色 2" xfId="31"/>
-    <cellStyle builtinId="36" name="60% - 强调文字颜色 2" xfId="32"/>
-    <cellStyle builtinId="37" name="强调文字颜色 3" xfId="33"/>
-    <cellStyle builtinId="38" name="20% - 强调文字颜色 3" xfId="34"/>
-    <cellStyle builtinId="39" name="40% - 强调文字颜色 3" xfId="35"/>
-    <cellStyle builtinId="40" name="60% - 强调文字颜色 3" xfId="36"/>
-    <cellStyle builtinId="41" name="强调文字颜色 4" xfId="37"/>
-    <cellStyle builtinId="42" name="20% - 强调文字颜色 4" xfId="38"/>
-    <cellStyle builtinId="43" name="40% - 强调文字颜色 4" xfId="39"/>
-    <cellStyle builtinId="44" name="60% - 强调文字颜色 4" xfId="40"/>
-    <cellStyle builtinId="45" name="强调文字颜色 5" xfId="41"/>
-    <cellStyle builtinId="46" name="20% - 强调文字颜色 5" xfId="42"/>
-    <cellStyle builtinId="47" name="40% - 强调文字颜色 5" xfId="43"/>
-    <cellStyle builtinId="48" name="60% - 强调文字颜色 5" xfId="44"/>
-    <cellStyle builtinId="49" name="强调文字颜色 6" xfId="45"/>
-    <cellStyle builtinId="50" name="20% - 强调文字颜色 6" xfId="46"/>
-    <cellStyle builtinId="51" name="40% - 强调文字颜色 6" xfId="47"/>
-    <cellStyle builtinId="52" name="60% - 强调文字颜色 6" xfId="48"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
     <cellStyle name="Normal" xfId="49"/>
   </cellStyles>
   <dxfs count="8">
@@ -1206,14 +1096,82 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="2" defaultPivotStyle="PivotStylePreset2_Accent1 1" defaultTableStyle="TableStylePreset3_Accent1">
-    <tableStyle count="7" name="TableStylePreset3_Accent1" pivot="0">
-      <tableStyleElement dxfId="0" type="firstColumnStripe"/>
+  <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle count="1" name="PivotStylePreset2_Accent1 1" table="0">
-      <tableStyleElement dxfId="7" type="pageFieldValues"/>
+    <tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="1">
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1370,73 +1328,112 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:R22"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.1"/>
   <cols>
-    <col customWidth="1" max="1" min="1" style="1" width="21.2166666666667"/>
-    <col customWidth="1" max="2" min="2" style="1" width="12.35"/>
-    <col customWidth="1" max="8" min="3" style="1" width="11.5"/>
-    <col customWidth="1" max="9" min="9" style="1" width="14.9333333333333"/>
-    <col customWidth="1" max="12" min="10" style="1" width="11.5"/>
+    <col width="21.2166666666667" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.35" customWidth="1" style="1" min="2" max="2"/>
+    <col width="11.5" customWidth="1" style="1" min="3" max="8"/>
+    <col width="14.9333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="1" min="10" max="12"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="44" r="1" s="1" spans="1:18">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+    <row r="1" ht="44" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
       </c>
       <c r="B1" s="3" t="n"/>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="22" r="2" s="1" spans="1:18">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>CIFAR100 (T=10)</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>CUB200 (T=10)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=5)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>OmniBenchmark (T=10)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>VTAB (T=5)</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="1">
       <c r="A2" s="7" t="n"/>
       <c r="B2" s="8" t="n"/>
-      <c r="C2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="3" s="1" spans="1:18">
-      <c r="A3" s="18" t="s">
-        <v>8</v>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Full Fine-Tuning</t>
+        </is>
       </c>
       <c r="B3" s="18" t="n"/>
       <c r="C3" s="18" t="n">
@@ -1470,12 +1467,16 @@
         <v>78.67</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="4" s="1" spans="1:18">
-      <c r="A4" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>10</v>
+    <row r="4" ht="20" customHeight="1" s="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C4" s="18" t="n">
         <v>81.28</v>
@@ -1508,12 +1509,16 @@
         <v>90.8</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="5" s="1" spans="1:18">
-      <c r="A5" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>10</v>
+    <row r="5" ht="20" customHeight="1" s="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>APER</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C5" s="18" t="n">
         <v>87.52</v>
@@ -1546,12 +1551,16 @@
         <v>90.81</v>
       </c>
     </row>
-    <row customHeight="1" ht="26" r="6" s="1" spans="1:18">
-      <c r="A6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>13</v>
+    <row r="6" ht="26" customHeight="1" s="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2022</t>
+        </is>
       </c>
       <c r="C6" s="18" t="n">
         <v>85.13</v>
@@ -1584,12 +1593,16 @@
         <v>81.7</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="7" s="1" spans="1:18">
-      <c r="A7" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>15</v>
+    <row r="7" ht="20" customHeight="1" s="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C7" s="19" t="n">
         <v>85.33</v>
@@ -1622,12 +1635,16 @@
         <v>89.90000000000001</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="8" s="1" spans="1:18">
-      <c r="A8" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>17</v>
+    <row r="8" ht="20" customHeight="1" s="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2023</t>
+        </is>
       </c>
       <c r="C8" s="20" t="n">
         <v>86.55</v>
@@ -1660,12 +1677,16 @@
         <v>87.23</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="9" s="1" spans="1:18">
-      <c r="A9" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>19</v>
+    <row r="9" ht="20" customHeight="1" s="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>LAE</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>ICCV 2023</t>
+        </is>
       </c>
       <c r="C9" s="18" t="n">
         <v>85.47</v>
@@ -1694,12 +1715,16 @@
         <v>85.62</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="10" s="1" spans="1:18">
-      <c r="A10" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>21</v>
+    <row r="10" ht="18.4" customHeight="1" s="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>InfLoRA</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C10" s="18" t="n">
         <v>86.27</v>
@@ -1728,12 +1753,16 @@
         <v>88.37</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="11" s="1" spans="1:18">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>21</v>
+    <row r="11" ht="18.4" customHeight="1" s="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>EASE</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C11" s="21" t="n">
         <v>88.13</v>
@@ -1766,12 +1795,16 @@
         <v>92.11</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="12" s="1" spans="1:18">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>24</v>
+    <row r="12" ht="18.4" customHeight="1" s="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>BiLoRA</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C12" s="21" t="n">
         <v>85.19</v>
@@ -1800,12 +1833,16 @@
       <c r="K12" s="21" t="n"/>
       <c r="L12" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="13" s="1" spans="1:18">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>26</v>
+    <row r="13" ht="18.4" customHeight="1" s="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>SD-LoRA</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>ICLR 2025</t>
+        </is>
       </c>
       <c r="C13" s="21" t="n">
         <v>87.58</v>
@@ -1838,12 +1875,16 @@
         <v>85.56</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="14" s="1" spans="1:18">
-      <c r="A14" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>24</v>
+    <row r="14" ht="18.4" customHeight="1" s="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>CL-LoRA</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C14" s="22" t="n">
         <v>88.06999999999999</v>
@@ -1876,7 +1917,7 @@
         <v>89.65000000000001</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="15" s="1" spans="1:18">
+    <row r="15" ht="18.4" customHeight="1" s="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="23" t="n"/>
@@ -1890,13 +1931,17 @@
       <c r="K15" s="23" t="n"/>
       <c r="L15" s="24" t="n"/>
     </row>
-    <row r="16" s="1" spans="1:18"/>
-    <row customHeight="1" ht="18.4" r="17" s="1" spans="1:18">
-      <c r="A17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>29</v>
+    <row r="16" s="1"/>
+    <row r="17" ht="18.4" customHeight="1" s="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>iCaRL</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>CVPR 2017</t>
+        </is>
       </c>
       <c r="C17" s="16" t="n">
         <v>72.52</v>
@@ -1920,16 +1965,22 @@
       </c>
       <c r="K17" s="16" t="n"/>
       <c r="L17" s="16" t="n"/>
-      <c r="M17" s="25" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="18.4" r="18" s="1" spans="1:18">
-      <c r="A18" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>15</v>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18.4" customHeight="1" s="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>FOSTER</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C18" s="16" t="n"/>
       <c r="D18" s="16" t="n"/>
@@ -1942,7 +1993,7 @@
       <c r="K18" s="16" t="n"/>
       <c r="L18" s="16" t="n"/>
     </row>
-    <row customHeight="1" ht="17.55" r="19" s="1" spans="1:18">
+    <row r="19" ht="17.55" customHeight="1" s="1">
       <c r="I19" s="26" t="n"/>
       <c r="J19" s="26" t="n"/>
       <c r="K19" s="26" t="n"/>
@@ -1954,7 +2005,7 @@
       <c r="Q19" s="26" t="n"/>
       <c r="R19" s="26" t="n"/>
     </row>
-    <row customHeight="1" ht="17.55" r="22" s="1" spans="1:18">
+    <row r="22" ht="17.55" customHeight="1" s="1">
       <c r="I22" s="26" t="n"/>
       <c r="J22" s="26" t="n"/>
       <c r="K22" s="26" t="n"/>
@@ -1975,7 +2026,7 @@
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1986,73 +2037,112 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1" defaultRowHeight="14.1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1" defaultRowHeight="14.1"/>
   <cols>
-    <col customWidth="1" max="1" min="1" style="1" width="21.2166666666667"/>
-    <col customWidth="1" max="2" min="2" style="1" width="12.35"/>
-    <col customWidth="1" max="8" min="3" style="1" width="11.5"/>
-    <col customWidth="1" max="9" min="9" style="1" width="14.9333333333333"/>
-    <col customWidth="1" max="12" min="10" style="1" width="11.5"/>
+    <col width="21.2166666666667" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.35" customWidth="1" style="1" min="2" max="2"/>
+    <col width="11.5" customWidth="1" style="1" min="3" max="8"/>
+    <col width="14.9333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="1" min="10" max="12"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="44" r="1" s="1" spans="1:13">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+    <row r="1" ht="44" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
       </c>
       <c r="B1" s="3" t="n"/>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="22" r="2" s="1" spans="1:13">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>CIFAR100 (T=10)</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>CUB200 (T=10)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=5)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>OmniBenchmark (T=10)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>VTAB (T=5)</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="1">
       <c r="A2" s="7" t="n"/>
       <c r="B2" s="8" t="n"/>
-      <c r="C2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="3" s="1" spans="1:13">
-      <c r="A3" s="18" t="s">
-        <v>8</v>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Full Fine-Tuning</t>
+        </is>
       </c>
       <c r="B3" s="18" t="n"/>
       <c r="C3" s="18" t="n">
@@ -2086,12 +2176,16 @@
         <v>68.02</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="4" s="1" spans="1:13">
-      <c r="A4" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>10</v>
+    <row r="4" ht="20" customHeight="1" s="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C4" s="18" t="n">
         <v>81.28</v>
@@ -2124,12 +2218,16 @@
         <v>90.45999999999999</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="5" s="1" spans="1:13">
-      <c r="A5" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>10</v>
+    <row r="5" ht="20" customHeight="1" s="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>APER</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C5" s="18" t="n">
         <v>88.25</v>
@@ -2162,12 +2260,16 @@
         <v>90.48999999999999</v>
       </c>
     </row>
-    <row customHeight="1" ht="26" r="6" s="1" spans="1:13">
-      <c r="A6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>13</v>
+    <row r="6" ht="26" customHeight="1" s="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2022</t>
+        </is>
       </c>
       <c r="C6" s="18" t="n">
         <v>85.27</v>
@@ -2200,12 +2302,16 @@
         <v>76.33</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="7" s="1" spans="1:13">
-      <c r="A7" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>15</v>
+    <row r="7" ht="20" customHeight="1" s="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C7" s="19" t="n">
         <v>85.39</v>
@@ -2238,12 +2344,16 @@
         <v>85.38</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="8" s="1" spans="1:13">
-      <c r="A8" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>17</v>
+    <row r="8" ht="20" customHeight="1" s="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2023</t>
+        </is>
       </c>
       <c r="C8" s="20" t="n">
         <v>87.68000000000001</v>
@@ -2276,12 +2386,16 @@
         <v>80.11</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="9" s="1" spans="1:13">
-      <c r="A9" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>19</v>
+    <row r="9" ht="20" customHeight="1" s="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>LAE</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>ICCV 2023</t>
+        </is>
       </c>
       <c r="C9" s="18" t="n">
         <v>85.56</v>
@@ -2310,12 +2424,16 @@
         <v>79.81999999999999</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="10" s="1" spans="1:13">
-      <c r="A10" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>21</v>
+    <row r="10" ht="18.4" customHeight="1" s="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>InfLoRA</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C10" s="18" t="n">
         <v>86.18000000000001</v>
@@ -2348,12 +2466,16 @@
         <v>84.86</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="11" s="1" spans="1:13">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>21</v>
+    <row r="11" ht="18.4" customHeight="1" s="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>EASE</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C11" s="21" t="n">
         <v>87.86</v>
@@ -2386,12 +2508,16 @@
         <v>85.66</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="12" s="1" spans="1:13">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>24</v>
+    <row r="12" ht="18.4" customHeight="1" s="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>BiLoRA</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C12" s="21" t="n">
         <v>86.27</v>
@@ -2416,12 +2542,16 @@
       <c r="K12" s="21" t="n"/>
       <c r="L12" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="13" s="1" spans="1:13">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>26</v>
+    <row r="13" ht="18.4" customHeight="1" s="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>SD-LoRA</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>ICLR 2025</t>
+        </is>
       </c>
       <c r="C13" s="21" t="n">
         <v>87.43000000000001</v>
@@ -2454,12 +2584,16 @@
         <v>86.67</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="14" s="1" spans="1:13">
-      <c r="A14" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>24</v>
+    <row r="14" ht="18.4" customHeight="1" s="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>CL-LoRA</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C14" s="22" t="n">
         <v>88.15000000000001</v>
@@ -2488,7 +2622,7 @@
       <c r="K14" s="22" t="n"/>
       <c r="L14" s="22" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="15" s="1" spans="1:13">
+    <row r="15" ht="18.4" customHeight="1" s="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="23" t="n"/>
@@ -2502,13 +2636,17 @@
       <c r="K15" s="23" t="n"/>
       <c r="L15" s="24" t="n"/>
     </row>
-    <row r="16" s="1" spans="1:13"/>
-    <row customHeight="1" ht="18.4" r="17" s="1" spans="1:13">
-      <c r="A17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>29</v>
+    <row r="16" s="1"/>
+    <row r="17" ht="18.4" customHeight="1" s="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>iCaRL</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>CVPR 2017</t>
+        </is>
       </c>
       <c r="C17" s="16" t="n">
         <v>73.51000000000001</v>
@@ -2532,16 +2670,22 @@
       </c>
       <c r="K17" s="16" t="n"/>
       <c r="L17" s="16" t="n"/>
-      <c r="M17" s="25" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="18.4" r="18" s="1" spans="1:13">
-      <c r="A18" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>15</v>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18.4" customHeight="1" s="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>FOSTER</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C18" s="16" t="n"/>
       <c r="D18" s="16" t="n"/>
@@ -2554,7 +2698,7 @@
       <c r="K18" s="16" t="n"/>
       <c r="L18" s="16" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="19" s="1" spans="1:13"/>
+    <row r="19" ht="18.4" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="C1:D1"/>
@@ -2564,7 +2708,7 @@
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -2575,73 +2719,112 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1" defaultRowHeight="14.1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1" defaultRowHeight="14.1"/>
   <cols>
-    <col customWidth="1" max="1" min="1" style="1" width="21.2166666666667"/>
-    <col customWidth="1" max="2" min="2" style="1" width="12.35"/>
-    <col customWidth="1" max="8" min="3" style="1" width="11.5"/>
-    <col customWidth="1" max="9" min="9" style="1" width="14.9333333333333"/>
-    <col customWidth="1" max="12" min="10" style="1" width="11.5"/>
+    <col width="21.2166666666667" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.35" customWidth="1" style="1" min="2" max="2"/>
+    <col width="11.5" customWidth="1" style="1" min="3" max="8"/>
+    <col width="14.9333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="1" min="10" max="12"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="44" r="1" s="1" spans="1:13">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+    <row r="1" ht="44" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
       </c>
       <c r="B1" s="3" t="n"/>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="22" r="2" s="1" spans="1:13">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>CIFAR100 (T=10)</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>CUB200 (T=10)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=5)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>OmniBenchmark (T=10)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>VTAB (T=5)</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="1">
       <c r="A2" s="7" t="n"/>
       <c r="B2" s="8" t="n"/>
-      <c r="C2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="3" s="1" spans="1:13">
-      <c r="A3" s="18" t="s">
-        <v>8</v>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Full Fine-Tuning</t>
+        </is>
       </c>
       <c r="B3" s="18" t="n"/>
       <c r="C3" s="18" t="n">
@@ -2675,12 +2858,16 @@
         <v>66.12</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="4" s="1" spans="1:13">
-      <c r="A4" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>10</v>
+    <row r="4" ht="20" customHeight="1" s="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C4" s="18" t="n">
         <v>81.28</v>
@@ -2713,12 +2900,16 @@
         <v>90.67</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="5" s="1" spans="1:13">
-      <c r="A5" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>10</v>
+    <row r="5" ht="20" customHeight="1" s="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>APER</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C5" s="18" t="n">
         <v>86.88</v>
@@ -2751,12 +2942,16 @@
         <v>90.54000000000001</v>
       </c>
     </row>
-    <row customHeight="1" ht="26" r="6" s="1" spans="1:13">
-      <c r="A6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>13</v>
+    <row r="6" ht="26" customHeight="1" s="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2022</t>
+        </is>
       </c>
       <c r="C6" s="18" t="n">
         <v>83.58</v>
@@ -2789,12 +2984,16 @@
         <v>79.16</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="7" s="1" spans="1:13">
-      <c r="A7" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>15</v>
+    <row r="7" ht="20" customHeight="1" s="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C7" s="19" t="n">
         <v>84.97</v>
@@ -2827,12 +3026,16 @@
         <v>85.83</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="8" s="1" spans="1:13">
-      <c r="A8" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>17</v>
+    <row r="8" ht="20" customHeight="1" s="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2023</t>
+        </is>
       </c>
       <c r="C8" s="20" t="n">
         <v>87.19</v>
@@ -2865,12 +3068,16 @@
         <v>82.89</v>
       </c>
     </row>
-    <row customHeight="1" ht="20" r="9" s="1" spans="1:13">
-      <c r="A9" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>19</v>
+    <row r="9" ht="20" customHeight="1" s="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>LAE</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>ICCV 2023</t>
+        </is>
       </c>
       <c r="C9" s="18" t="n">
         <v>85.01000000000001</v>
@@ -2884,8 +3091,12 @@
       <c r="F9" s="18" t="n">
         <v>80.2</v>
       </c>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
+      <c r="G9" s="18" t="n">
+        <v>71.13</v>
+      </c>
+      <c r="H9" s="18" t="n">
+        <v>75.09</v>
+      </c>
       <c r="I9" s="18" t="n">
         <v>66.08</v>
       </c>
@@ -2899,12 +3110,16 @@
         <v>86.14</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="10" s="1" spans="1:13">
-      <c r="A10" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>21</v>
+    <row r="10" ht="18.4" customHeight="1" s="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>InfLoRA</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C10" s="18" t="n">
         <v>87.06</v>
@@ -2937,12 +3152,16 @@
         <v>87.73</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="11" s="1" spans="1:13">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>21</v>
+    <row r="11" ht="18.4" customHeight="1" s="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>EASE</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C11" s="21" t="n">
         <v>88.04000000000001</v>
@@ -2975,12 +3194,16 @@
         <v>90.72</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="12" s="1" spans="1:13">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>24</v>
+    <row r="12" ht="18.4" customHeight="1" s="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>BiLoRA</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C12" s="21" t="n">
         <v>85.94</v>
@@ -3005,12 +3228,16 @@
       <c r="K12" s="21" t="n"/>
       <c r="L12" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="13" s="1" spans="1:13">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>26</v>
+    <row r="13" ht="18.4" customHeight="1" s="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>SD-LoRA</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>ICLR 2025</t>
+        </is>
       </c>
       <c r="C13" s="21" t="n"/>
       <c r="D13" s="21" t="n"/>
@@ -3039,12 +3266,16 @@
         <v>84.93000000000001</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="14" s="1" spans="1:13">
-      <c r="A14" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>24</v>
+    <row r="14" ht="18.4" customHeight="1" s="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>CL-LoRA</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C14" s="22" t="n">
         <v>86.09</v>
@@ -3073,7 +3304,7 @@
       <c r="K14" s="22" t="n"/>
       <c r="L14" s="22" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="15" s="1" spans="1:13">
+    <row r="15" ht="18.4" customHeight="1" s="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="23" t="n"/>
@@ -3087,13 +3318,17 @@
       <c r="K15" s="23" t="n"/>
       <c r="L15" s="24" t="n"/>
     </row>
-    <row r="16" s="1" spans="1:13"/>
-    <row customHeight="1" ht="18.4" r="17" s="1" spans="1:13">
-      <c r="A17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>29</v>
+    <row r="16" s="1"/>
+    <row r="17" ht="18.4" customHeight="1" s="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>iCaRL</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>CVPR 2017</t>
+        </is>
       </c>
       <c r="C17" s="16" t="n">
         <v>72.69</v>
@@ -3117,16 +3352,22 @@
       </c>
       <c r="K17" s="16" t="n"/>
       <c r="L17" s="16" t="n"/>
-      <c r="M17" s="25" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="18.4" r="18" s="1" spans="1:13">
-      <c r="A18" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>15</v>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18.4" customHeight="1" s="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>FOSTER</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C18" s="16" t="n"/>
       <c r="D18" s="16" t="n"/>
@@ -3139,7 +3380,7 @@
       <c r="K18" s="16" t="n"/>
       <c r="L18" s="16" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="19" s="1" spans="1:13"/>
+    <row r="19" ht="18.4" customHeight="1" s="1"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="C1:D1"/>
@@ -3149,7 +3390,7 @@
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -3160,73 +3401,112 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1" defaultRowHeight="14.1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9.1" defaultRowHeight="14.1"/>
   <cols>
-    <col customWidth="1" max="1" min="1" style="1" width="21.2166666666667"/>
-    <col customWidth="1" max="2" min="2" style="1" width="12.35"/>
-    <col customWidth="1" max="8" min="3" style="1" width="11.5"/>
-    <col customWidth="1" max="9" min="9" style="1" width="14.9333333333333"/>
-    <col customWidth="1" max="12" min="10" style="1" width="11.5"/>
+    <col width="21.2166666666667" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.35" customWidth="1" style="1" min="2" max="2"/>
+    <col width="11.5" customWidth="1" style="1" min="3" max="8"/>
+    <col width="14.9333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="1" min="10" max="12"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="44" r="1" s="1" spans="1:13">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+    <row r="1" ht="44" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
       </c>
       <c r="B1" s="3" t="n"/>
-      <c r="C1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="13" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="22" r="2" s="1" spans="1:13">
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>CIFAR100 (T=10)</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>CUB200 (T=10)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=5)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>OmniBenchmark (T=10)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>VTAB (T=5)</t>
+        </is>
+      </c>
+      <c r="L1" s="14" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1" s="1">
       <c r="A2" s="7" t="n"/>
       <c r="B2" s="8" t="n"/>
-      <c r="C2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="L2" s="15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="20" r="3" s="1" spans="1:13">
-      <c r="A3" s="18" t="s">
-        <v>8</v>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="L2" s="15" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" s="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Full Fine-Tuning</t>
+        </is>
       </c>
       <c r="B3" s="18" t="n"/>
       <c r="C3" s="18" t="n"/>
@@ -3240,12 +3520,16 @@
       <c r="K3" s="18" t="n"/>
       <c r="L3" s="18" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="4" s="1" spans="1:13">
-      <c r="A4" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>10</v>
+    <row r="4" ht="20" customHeight="1" s="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C4" s="18" t="n"/>
       <c r="D4" s="18" t="n"/>
@@ -3258,12 +3542,16 @@
       <c r="K4" s="18" t="n"/>
       <c r="L4" s="18" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="5" s="1" spans="1:13">
-      <c r="A5" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>10</v>
+    <row r="5" ht="20" customHeight="1" s="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>APER</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>IJCV 2024</t>
+        </is>
       </c>
       <c r="C5" s="18" t="n"/>
       <c r="D5" s="18" t="n"/>
@@ -3276,12 +3564,16 @@
       <c r="K5" s="18" t="n"/>
       <c r="L5" s="18" t="n"/>
     </row>
-    <row customHeight="1" ht="26" r="6" s="1" spans="1:13">
-      <c r="A6" s="18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>13</v>
+    <row r="6" ht="26" customHeight="1" s="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>L2P</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2022</t>
+        </is>
       </c>
       <c r="C6" s="18" t="n"/>
       <c r="D6" s="18" t="n"/>
@@ -3294,12 +3586,16 @@
       <c r="K6" s="18" t="n"/>
       <c r="L6" s="18" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="7" s="1" spans="1:13">
-      <c r="A7" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>15</v>
+    <row r="7" ht="20" customHeight="1" s="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>DualPrompt</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C7" s="19" t="n"/>
       <c r="D7" s="19" t="n"/>
@@ -3312,12 +3608,16 @@
       <c r="K7" s="19" t="n"/>
       <c r="L7" s="19" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="8" s="1" spans="1:13">
-      <c r="A8" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>17</v>
+    <row r="8" ht="20" customHeight="1" s="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>CODA-Prompt</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2023</t>
+        </is>
       </c>
       <c r="C8" s="20" t="n"/>
       <c r="D8" s="20" t="n"/>
@@ -3330,12 +3630,16 @@
       <c r="K8" s="20" t="n"/>
       <c r="L8" s="20" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="9" s="1" spans="1:13">
-      <c r="A9" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>19</v>
+    <row r="9" ht="20" customHeight="1" s="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>LAE</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>ICCV 2023</t>
+        </is>
       </c>
       <c r="C9" s="18" t="n"/>
       <c r="D9" s="18" t="n"/>
@@ -3348,12 +3652,16 @@
       <c r="K9" s="18" t="n"/>
       <c r="L9" s="18" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="10" s="1" spans="1:13">
-      <c r="A10" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>21</v>
+    <row r="10" ht="18.4" customHeight="1" s="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>InfLoRA</t>
+        </is>
+      </c>
+      <c r="B10" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C10" s="18" t="n"/>
       <c r="D10" s="18" t="n"/>
@@ -3366,12 +3674,16 @@
       <c r="K10" s="18" t="n"/>
       <c r="L10" s="18" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="11" s="1" spans="1:13">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>21</v>
+    <row r="11" ht="18.4" customHeight="1" s="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>EASE</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C11" s="21" t="n"/>
       <c r="D11" s="21" t="n"/>
@@ -3384,12 +3696,16 @@
       <c r="K11" s="21" t="n"/>
       <c r="L11" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="12" s="1" spans="1:13">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>24</v>
+    <row r="12" ht="18.4" customHeight="1" s="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>BiLoRA</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C12" s="21" t="n"/>
       <c r="D12" s="21" t="n"/>
@@ -3402,12 +3718,16 @@
       <c r="K12" s="21" t="n"/>
       <c r="L12" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="13" s="1" spans="1:13">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>26</v>
+    <row r="13" ht="18.4" customHeight="1" s="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>SD-LoRA</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>ICLR 2025</t>
+        </is>
       </c>
       <c r="C13" s="21" t="n"/>
       <c r="D13" s="21" t="n"/>
@@ -3420,12 +3740,16 @@
       <c r="K13" s="21" t="n"/>
       <c r="L13" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="14" s="1" spans="1:13">
-      <c r="A14" s="18" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>24</v>
+    <row r="14" ht="18.4" customHeight="1" s="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>CL-LoRA</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C14" s="22" t="n">
         <v>86.44</v>
@@ -3458,7 +3782,7 @@
         <v>80.05</v>
       </c>
     </row>
-    <row customHeight="1" ht="18.4" r="15" s="1" spans="1:13">
+    <row r="15" ht="18.4" customHeight="1" s="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="23" t="n"/>
@@ -3472,13 +3796,17 @@
       <c r="K15" s="23" t="n"/>
       <c r="L15" s="24" t="n"/>
     </row>
-    <row r="16" s="1" spans="1:13"/>
-    <row customHeight="1" ht="18.4" r="17" s="1" spans="1:13">
-      <c r="A17" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>29</v>
+    <row r="16" s="1"/>
+    <row r="17" ht="18.4" customHeight="1" s="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>iCaRL</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>CVPR 2017</t>
+        </is>
       </c>
       <c r="C17" s="16" t="n"/>
       <c r="D17" s="16" t="n"/>
@@ -3490,16 +3818,22 @@
       <c r="J17" s="16" t="n"/>
       <c r="K17" s="16" t="n"/>
       <c r="L17" s="16" t="n"/>
-      <c r="M17" s="25" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row customHeight="1" ht="18.4" r="18" s="1" spans="1:13">
-      <c r="A18" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>15</v>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>Memory</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18.4" customHeight="1" s="1">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>FOSTER</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>ECCV 2022</t>
+        </is>
       </c>
       <c r="C18" s="16" t="n"/>
       <c r="D18" s="16" t="n"/>
@@ -3521,7 +3855,7 @@
     <mergeCell ref="K1:L1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -3532,70 +3866,102 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L18"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.1"/>
   <cols>
-    <col customWidth="1" max="1" min="1" style="1" width="21.2166666666667"/>
-    <col customWidth="1" max="2" min="2" style="1" width="12.35"/>
-    <col customWidth="1" max="8" min="3" style="1" width="11.5"/>
-    <col customWidth="1" max="9" min="9" style="1" width="14.9333333333333"/>
-    <col customWidth="1" max="12" min="10" style="1" width="11.5"/>
-    <col customWidth="1" max="13" min="13" style="1" width="22.9166666666667"/>
-    <col customWidth="1" max="14" min="14" style="1" width="17.4"/>
+    <col width="21.2166666666667" customWidth="1" style="1" min="1" max="1"/>
+    <col width="12.35" customWidth="1" style="1" min="2" max="2"/>
+    <col width="11.5" customWidth="1" style="1" min="3" max="8"/>
+    <col width="14.9333333333333" customWidth="1" style="1" min="9" max="9"/>
+    <col width="11.5" customWidth="1" style="1" min="10" max="12"/>
+    <col width="22.9166666666667" customWidth="1" style="1" min="13" max="13"/>
+    <col width="17.4" customWidth="1" style="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row customHeight="1" ht="44" r="1" s="1" spans="1:12">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
+    <row r="1" ht="44" customHeight="1" s="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
       </c>
       <c r="B1" s="3" t="n"/>
-      <c r="C1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>34</v>
-      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=5)</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="n"/>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=10)</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=20)</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="n"/>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>ImageNet-R (T=40)</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="n"/>
       <c r="K1" s="6" t="n"/>
       <c r="L1" s="6" t="n"/>
     </row>
-    <row customHeight="1" ht="22" r="2" s="1" spans="1:12">
+    <row r="2" ht="22" customHeight="1" s="1">
       <c r="A2" s="7" t="n"/>
       <c r="B2" s="8" t="n"/>
-      <c r="C2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H2" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="I2" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J2" s="9" t="s">
-        <v>7</v>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>A_L</t>
+        </is>
+      </c>
+      <c r="J2" s="9" t="inlineStr">
+        <is>
+          <t>Ā</t>
+        </is>
       </c>
       <c r="K2" s="6" t="n"/>
       <c r="L2" s="6" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="3" s="1" spans="1:12">
-      <c r="A3" s="18" t="s">
-        <v>8</v>
+    <row r="3" ht="20" customHeight="1" s="1">
+      <c r="A3" s="18" t="inlineStr">
+        <is>
+          <t>Full Fine-Tuning</t>
+        </is>
       </c>
       <c r="B3" s="18" t="n"/>
       <c r="C3" s="18" t="n"/>
@@ -3609,9 +3975,11 @@
       <c r="K3" s="10" t="n"/>
       <c r="L3" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="4" s="1" spans="1:12">
-      <c r="A4" s="18" t="s">
-        <v>9</v>
+    <row r="4" ht="20" customHeight="1" s="1">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>SimpleCIL</t>
+        </is>
       </c>
       <c r="B4" s="18" t="n"/>
       <c r="C4" s="18" t="n"/>
@@ -3625,9 +3993,11 @@
       <c r="K4" s="10" t="n"/>
       <c r="L4" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="5" s="1" spans="1:12">
-      <c r="A5" s="18" t="s">
-        <v>11</v>
+    <row r="5" ht="20" customHeight="1" s="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>APER</t>
+        </is>
       </c>
       <c r="B5" s="18" t="n"/>
       <c r="C5" s="18" t="n"/>
@@ -3641,7 +4011,7 @@
       <c r="K5" s="10" t="n"/>
       <c r="L5" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="26" r="6" s="1" spans="1:12">
+    <row r="6" ht="26" customHeight="1" s="1">
       <c r="A6" s="18" t="n"/>
       <c r="B6" s="18" t="n"/>
       <c r="C6" s="18" t="n"/>
@@ -3655,7 +4025,7 @@
       <c r="K6" s="10" t="n"/>
       <c r="L6" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="7" s="1" spans="1:12">
+    <row r="7" ht="20" customHeight="1" s="1">
       <c r="A7" s="18" t="n"/>
       <c r="B7" s="18" t="n"/>
       <c r="C7" s="19" t="n"/>
@@ -3669,7 +4039,7 @@
       <c r="K7" s="10" t="n"/>
       <c r="L7" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="8" s="1" spans="1:12">
+    <row r="8" ht="20" customHeight="1" s="1">
       <c r="A8" s="18" t="n"/>
       <c r="B8" s="18" t="n"/>
       <c r="C8" s="20" t="n"/>
@@ -3683,9 +4053,11 @@
       <c r="K8" s="12" t="n"/>
       <c r="L8" s="12" t="n"/>
     </row>
-    <row customHeight="1" ht="20" r="9" s="1" spans="1:12">
-      <c r="A9" s="18" t="s">
-        <v>18</v>
+    <row r="9" ht="20" customHeight="1" s="1">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>LAE</t>
+        </is>
       </c>
       <c r="B9" s="18" t="n"/>
       <c r="C9" s="18" t="n"/>
@@ -3699,9 +4071,11 @@
       <c r="K9" s="12" t="n"/>
       <c r="L9" s="12" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="10" s="1" spans="1:12">
-      <c r="A10" s="18" t="s">
-        <v>20</v>
+    <row r="10" ht="18.4" customHeight="1" s="1">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>InfLoRA</t>
+        </is>
       </c>
       <c r="B10" s="18" t="n"/>
       <c r="C10" s="18" t="n">
@@ -3719,12 +4093,16 @@
       <c r="K10" s="10" t="n"/>
       <c r="L10" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="11" s="1" spans="1:12">
-      <c r="A11" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>21</v>
+    <row r="11" ht="18.4" customHeight="1" s="1">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>EASE</t>
+        </is>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2024</t>
+        </is>
       </c>
       <c r="C11" s="21" t="n"/>
       <c r="D11" s="21" t="n"/>
@@ -3737,12 +4115,16 @@
       <c r="K11" s="10" t="n"/>
       <c r="L11" s="10" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="12" s="1" spans="1:12">
-      <c r="A12" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="21" t="s">
-        <v>24</v>
+    <row r="12" ht="18.4" customHeight="1" s="1">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>BiLoRA</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>CVPR 2025</t>
+        </is>
       </c>
       <c r="C12" s="21" t="n">
         <v>76.33</v>
@@ -3757,12 +4139,16 @@
       <c r="I12" s="21" t="n"/>
       <c r="J12" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="13" s="1" spans="1:12">
-      <c r="A13" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>26</v>
+    <row r="13" ht="18.4" customHeight="1" s="1">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>SD-LoRA</t>
+        </is>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>ICLR 2025</t>
+        </is>
       </c>
       <c r="C13" s="21" t="n"/>
       <c r="D13" s="21" t="n"/>
@@ -3773,9 +4159,11 @@
       <c r="I13" s="21" t="n"/>
       <c r="J13" s="21" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="14" s="1" spans="1:12">
-      <c r="A14" s="18" t="s">
-        <v>27</v>
+    <row r="14" ht="18.4" customHeight="1" s="1">
+      <c r="A14" s="18" t="inlineStr">
+        <is>
+          <t>CL-LoRA</t>
+        </is>
       </c>
       <c r="B14" s="18" t="n"/>
       <c r="C14" s="22" t="n"/>
@@ -3787,7 +4175,7 @@
       <c r="I14" s="22" t="n"/>
       <c r="J14" s="22" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="15" s="1" spans="1:12">
+    <row r="15" ht="18.4" customHeight="1" s="1">
       <c r="A15" s="10" t="n"/>
       <c r="B15" s="10" t="n"/>
       <c r="C15" s="23" t="n"/>
@@ -3799,8 +4187,8 @@
       <c r="I15" s="23" t="n"/>
       <c r="J15" s="23" t="n"/>
     </row>
-    <row r="16" s="1" spans="1:12"/>
-    <row customHeight="1" ht="18.4" r="17" s="1" spans="1:12">
+    <row r="16" s="1"/>
+    <row r="17" ht="18.4" customHeight="1" s="1">
       <c r="A17" s="16" t="n"/>
       <c r="B17" s="16" t="n"/>
       <c r="C17" s="16" t="n"/>
@@ -3812,7 +4200,7 @@
       <c r="I17" s="16" t="n"/>
       <c r="J17" s="16" t="n"/>
     </row>
-    <row customHeight="1" ht="18.4" r="18" s="1" spans="1:12">
+    <row r="18" ht="18.4" customHeight="1" s="1">
       <c r="A18" s="16" t="n"/>
       <c r="B18" s="16" t="n"/>
       <c r="C18" s="16" t="n"/>
@@ -3831,6 +4219,6 @@
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="I1:J1"/>
   </mergeCells>
-  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>